<commit_message>
Change min max VO2Max & Min HRR
</commit_message>
<xml_diff>
--- a/Lab4_BVT.xlsx
+++ b/Lab4_BVT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\than\Downloads\KKU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\SQA\Lab4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E015D4FB-4B99-49F7-8779-0EDBD581B3A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0696BBE3-6B3F-4D41-900B-2E87911D6A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="72">
   <si>
     <t>Test Case Design and Test Results</t>
   </si>
@@ -245,16 +245,16 @@
     <t>ธนภูมิ แทนทุมมา</t>
   </si>
   <si>
-    <t>ค่า RHR ต่ำกว่าค่ากำหนด</t>
-  </si>
-  <si>
-    <t>ค่า RHR เกินกว่าค่ากำหนด</t>
-  </si>
-  <si>
-    <t>ค่า HRR สูงกว่ากำหนด</t>
-  </si>
-  <si>
     <t>java 26.0.1 2026-04-21, window 11</t>
+  </si>
+  <si>
+    <t>ค่า VO2 Max ไม่อยู่ในขอบเขต</t>
+  </si>
+  <si>
+    <t>ค่า RHR ไม่อยู่ในขอบเขตค่าที่กำหนด</t>
+  </si>
+  <si>
+    <t>ค่า HRR ไม่อยู่ในขอบเขตค่าที่กำหนด</t>
   </si>
 </sst>
 </file>
@@ -316,13 +316,13 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="18"/>
+      <sz val="16"/>
+      <color theme="1"/>
       <name val="TH SarabunPSK"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="16"/>
-      <color theme="1"/>
       <name val="TH SarabunPSK"/>
       <family val="2"/>
     </font>
@@ -510,6 +510,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -543,8 +545,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -987,15 +987,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="27"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
         <v>63</v>
@@ -1013,25 +1013,25 @@
         <v>11</v>
       </c>
       <c r="K2" s="6">
-        <v>24</v>
+        <v>-1</v>
       </c>
       <c r="L2" s="1">
         <v>39</v>
       </c>
       <c r="M2" s="6">
-        <v>11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
@@ -1042,25 +1042,25 @@
         <v>10</v>
       </c>
       <c r="K3" s="6">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L3" s="6">
         <v>40</v>
       </c>
       <c r="M3" s="6">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1071,42 +1071,42 @@
         <v>9</v>
       </c>
       <c r="K4" s="6">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="L4" s="6">
         <v>41</v>
       </c>
       <c r="M4" s="6">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="30"/>
+      <c r="B5" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="32"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="34">
+      <c r="G5" s="23">
         <v>244544</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K5" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="L5" s="6">
         <v>130</v>
       </c>
       <c r="M5" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.75">
@@ -1114,7 +1114,7 @@
         <v>7</v>
       </c>
       <c r="K6" s="6">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="L6" s="6">
         <v>219</v>
@@ -1124,28 +1124,28 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="25.05" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="31" t="s">
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="33" t="s">
+      <c r="F7" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="35" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="K7" s="6">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L7" s="6">
         <v>220</v>
@@ -1155,7 +1155,7 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A8" s="31"/>
+      <c r="A8" s="33"/>
       <c r="B8" s="8" t="s">
         <v>63</v>
       </c>
@@ -1165,14 +1165,14 @@
       <c r="D8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="35"/>
       <c r="J8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="K8" s="6">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L8" s="6">
         <v>221</v>
@@ -1186,17 +1186,17 @@
         <v>44</v>
       </c>
       <c r="B9" s="6">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C9" s="6">
         <v>130</v>
       </c>
       <c r="D9" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E9" s="6">
-        <f>1+1+4</f>
-        <v>6</v>
+        <f>0+1+3</f>
+        <v>4</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
@@ -1206,17 +1206,17 @@
         <v>45</v>
       </c>
       <c r="B10" s="6">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C10" s="6">
         <v>130</v>
       </c>
       <c r="D10" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E10" s="6">
-        <f>1+1+4</f>
-        <v>6</v>
+        <f>0+1+3</f>
+        <v>4</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
@@ -1226,17 +1226,17 @@
         <v>46</v>
       </c>
       <c r="B11" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C11" s="6">
         <v>130</v>
       </c>
       <c r="D11" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E11" s="6">
-        <f>3+1+6</f>
-        <v>10</v>
+        <f>2+1+3</f>
+        <v>6</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -1250,17 +1250,17 @@
         <v>47</v>
       </c>
       <c r="B12" s="6">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C12" s="6">
         <v>130</v>
       </c>
       <c r="D12" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E12" s="6">
-        <f>4+1+4</f>
-        <v>9</v>
+        <f>4+1+3</f>
+        <v>8</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
@@ -1274,16 +1274,16 @@
         <v>48</v>
       </c>
       <c r="B13" s="6">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C13" s="6">
         <v>130</v>
       </c>
       <c r="D13" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E13" s="6">
-        <f>4+1+4</f>
+        <f>5+1+3</f>
         <v>9</v>
       </c>
       <c r="F13" s="6"/>
@@ -1298,17 +1298,17 @@
         <v>49</v>
       </c>
       <c r="B14" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C14" s="6">
         <v>40</v>
       </c>
       <c r="D14" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E14" s="6">
-        <f>3+5+4</f>
-        <v>12</v>
+        <f>2+5+3</f>
+        <v>10</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
@@ -1322,17 +1322,17 @@
         <v>50</v>
       </c>
       <c r="B15" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C15" s="6">
         <v>41</v>
       </c>
       <c r="D15" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E15" s="6">
-        <f>3+5+4</f>
-        <v>12</v>
+        <f>2+5+3</f>
+        <v>10</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
@@ -1346,17 +1346,17 @@
         <v>51</v>
       </c>
       <c r="B16" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C16" s="6">
         <v>219</v>
       </c>
       <c r="D16" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E16" s="6">
-        <f>3+1+4</f>
-        <v>8</v>
+        <f>2+1+3</f>
+        <v>6</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
@@ -1370,17 +1370,17 @@
         <v>52</v>
       </c>
       <c r="B17" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C17" s="6">
         <v>220</v>
       </c>
       <c r="D17" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E17" s="6">
-        <f>3+1+4</f>
-        <v>8</v>
+        <f>2+1+3</f>
+        <v>6</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
@@ -1391,17 +1391,17 @@
         <v>53</v>
       </c>
       <c r="B18" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C18" s="6">
         <v>130</v>
       </c>
       <c r="D18" s="6">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E18" s="6">
-        <f>3+1+3</f>
-        <v>7</v>
+        <f>2+1+1</f>
+        <v>4</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="6"/>
@@ -1415,17 +1415,17 @@
         <v>54</v>
       </c>
       <c r="B19" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C19" s="6">
         <v>130</v>
       </c>
       <c r="D19" s="6">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E19" s="6">
-        <f>3+1+3</f>
-        <v>7</v>
+        <f>2+1+1</f>
+        <v>4</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
@@ -1435,7 +1435,7 @@
         <v>55</v>
       </c>
       <c r="B20" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C20" s="6">
         <v>130</v>
@@ -1444,8 +1444,8 @@
         <v>29</v>
       </c>
       <c r="E20" s="6">
-        <f>3+1+5</f>
-        <v>9</v>
+        <f>2+1+5</f>
+        <v>8</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
@@ -1455,7 +1455,7 @@
         <v>56</v>
       </c>
       <c r="B21" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C21" s="6">
         <v>130</v>
@@ -1464,8 +1464,8 @@
         <v>30</v>
       </c>
       <c r="E21" s="6">
-        <f>3+1+5</f>
-        <v>9</v>
+        <f>2+1+5</f>
+        <v>8</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
@@ -1536,7 +1536,7 @@
   <cols>
     <col min="1" max="1" width="19.796875" style="1" customWidth="1"/>
     <col min="2" max="4" width="21.296875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="32" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="45.5" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.19921875" style="1" customWidth="1"/>
     <col min="7" max="7" width="25.19921875" style="1" customWidth="1"/>
     <col min="8" max="10" width="10.796875" style="1"/>
@@ -1547,15 +1547,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="27"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
         <v>63</v>
@@ -1573,25 +1573,25 @@
         <v>11</v>
       </c>
       <c r="K2" s="6">
-        <v>24</v>
+        <v>-1</v>
       </c>
       <c r="L2" s="1">
         <v>39</v>
       </c>
       <c r="M2" s="6">
-        <v>11</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
@@ -1602,25 +1602,25 @@
         <v>10</v>
       </c>
       <c r="K3" s="6">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L3" s="6">
         <v>40</v>
       </c>
       <c r="M3" s="6">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1631,42 +1631,42 @@
         <v>9</v>
       </c>
       <c r="K4" s="6">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="L4" s="6">
         <v>41</v>
       </c>
       <c r="M4" s="6">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="30"/>
+      <c r="B5" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="32"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="34">
+      <c r="G5" s="23">
         <v>244544</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K5" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="L5" s="6">
         <v>130</v>
       </c>
       <c r="M5" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.75">
@@ -1674,7 +1674,7 @@
         <v>7</v>
       </c>
       <c r="K6" s="6">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="L6" s="6">
         <v>219</v>
@@ -1684,28 +1684,28 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="25.05" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="31" t="s">
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="31" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="33" t="s">
+      <c r="F7" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="35" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="K7" s="6">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L7" s="6">
         <v>220</v>
@@ -1715,7 +1715,7 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A8" s="31"/>
+      <c r="A8" s="33"/>
       <c r="B8" s="8" t="s">
         <v>63</v>
       </c>
@@ -1725,14 +1725,14 @@
       <c r="D8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="35"/>
       <c r="J8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="K8" s="6">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L8" s="6">
         <v>221</v>
@@ -1746,17 +1746,16 @@
         <v>44</v>
       </c>
       <c r="B9" s="6">
-        <v>24</v>
+        <v>-1</v>
       </c>
       <c r="C9" s="6">
         <v>130</v>
       </c>
       <c r="D9" s="6">
-        <v>21</v>
-      </c>
-      <c r="E9" s="35">
-        <f>0+1+4</f>
-        <v>5</v>
+        <v>15</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>69</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
@@ -1766,17 +1765,17 @@
         <v>45</v>
       </c>
       <c r="B10" s="6">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C10" s="6">
         <v>130</v>
       </c>
       <c r="D10" s="6">
-        <v>21</v>
-      </c>
-      <c r="E10" s="35">
-        <f>1+1+4</f>
-        <v>6</v>
+        <v>15</v>
+      </c>
+      <c r="E10" s="6">
+        <f>0+1+3</f>
+        <v>4</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
@@ -1786,17 +1785,17 @@
         <v>46</v>
       </c>
       <c r="B11" s="6">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C11" s="6">
         <v>130</v>
       </c>
       <c r="D11" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E11" s="6">
-        <f>1+1+4</f>
-        <v>6</v>
+        <f>0+1+3</f>
+        <v>4</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
@@ -1810,17 +1809,17 @@
         <v>47</v>
       </c>
       <c r="B12" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C12" s="6">
         <v>130</v>
       </c>
       <c r="D12" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E12" s="6">
-        <f>3+1+6</f>
-        <v>10</v>
+        <f>2+1+3</f>
+        <v>6</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
@@ -1834,17 +1833,17 @@
         <v>48</v>
       </c>
       <c r="B13" s="6">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C13" s="6">
         <v>130</v>
       </c>
       <c r="D13" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E13" s="6">
-        <f>4+1+4</f>
-        <v>9</v>
+        <f>4+1+3</f>
+        <v>8</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
@@ -1858,16 +1857,16 @@
         <v>49</v>
       </c>
       <c r="B14" s="6">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C14" s="6">
         <v>130</v>
       </c>
       <c r="D14" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E14" s="6">
-        <f>4+1+4</f>
+        <f>5+1+3</f>
         <v>9</v>
       </c>
       <c r="F14" s="6"/>
@@ -1882,17 +1881,17 @@
         <v>50</v>
       </c>
       <c r="B15" s="6">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C15" s="6">
         <v>130</v>
       </c>
       <c r="D15" s="6">
-        <v>21</v>
-      </c>
-      <c r="E15" s="35">
-        <f>5+1+4</f>
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="E15" s="6">
+        <f>5+1+3</f>
+        <v>9</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
@@ -1906,16 +1905,16 @@
         <v>51</v>
       </c>
       <c r="B16" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C16" s="6">
         <v>39</v>
       </c>
       <c r="D16" s="6">
-        <v>21</v>
-      </c>
-      <c r="E16" s="36" t="s">
-        <v>68</v>
+        <v>15</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>70</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
@@ -1929,17 +1928,17 @@
         <v>52</v>
       </c>
       <c r="B17" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C17" s="6">
         <v>40</v>
       </c>
       <c r="D17" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E17" s="6">
-        <f>3+5+4</f>
-        <v>12</v>
+        <f>2+5+3</f>
+        <v>10</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
@@ -1950,17 +1949,17 @@
         <v>53</v>
       </c>
       <c r="B18" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C18" s="6">
         <v>41</v>
       </c>
       <c r="D18" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E18" s="6">
-        <f>3+5+4</f>
-        <v>12</v>
+        <f>2+5+3</f>
+        <v>10</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="6"/>
@@ -1974,17 +1973,17 @@
         <v>54</v>
       </c>
       <c r="B19" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C19" s="6">
         <v>219</v>
       </c>
       <c r="D19" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E19" s="6">
-        <f>3+1+4</f>
-        <v>8</v>
+        <f>2+1+3</f>
+        <v>6</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
@@ -1994,17 +1993,17 @@
         <v>55</v>
       </c>
       <c r="B20" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C20" s="6">
         <v>220</v>
       </c>
       <c r="D20" s="6">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E20" s="6">
-        <f>3+1+4</f>
-        <v>8</v>
+        <f>2+1+3</f>
+        <v>6</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
@@ -2014,16 +2013,16 @@
         <v>56</v>
       </c>
       <c r="B21" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C21" s="6">
         <v>221</v>
       </c>
       <c r="D21" s="6">
-        <v>21</v>
-      </c>
-      <c r="E21" s="36" t="s">
-        <v>69</v>
+        <v>15</v>
+      </c>
+      <c r="E21" s="24" t="s">
+        <v>70</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6"/>
@@ -2037,17 +2036,16 @@
         <v>57</v>
       </c>
       <c r="B22" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C22" s="6">
         <v>130</v>
       </c>
       <c r="D22" s="6">
-        <v>11</v>
-      </c>
-      <c r="E22" s="6">
-        <f>3+1+1</f>
-        <v>5</v>
+        <v>-1</v>
+      </c>
+      <c r="E22" s="24" t="s">
+        <v>71</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
@@ -2061,17 +2059,17 @@
         <v>58</v>
       </c>
       <c r="B23" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C23" s="6">
         <v>130</v>
       </c>
       <c r="D23" s="6">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E23" s="6">
-        <f>3+1+3</f>
-        <v>7</v>
+        <f>2+1+1</f>
+        <v>4</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
@@ -2085,17 +2083,17 @@
         <v>59</v>
       </c>
       <c r="B24" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C24" s="6">
         <v>130</v>
       </c>
       <c r="D24" s="6">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E24" s="6">
-        <f>3+1+3</f>
-        <v>7</v>
+        <f>2+1+1</f>
+        <v>4</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
@@ -2109,7 +2107,7 @@
         <v>60</v>
       </c>
       <c r="B25" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C25" s="6">
         <v>130</v>
@@ -2118,8 +2116,8 @@
         <v>29</v>
       </c>
       <c r="E25" s="6">
-        <f>3+1+5</f>
-        <v>9</v>
+        <f>2+1+5</f>
+        <v>8</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
@@ -2133,7 +2131,7 @@
         <v>61</v>
       </c>
       <c r="B26" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C26" s="6">
         <v>130</v>
@@ -2142,8 +2140,8 @@
         <v>30</v>
       </c>
       <c r="E26" s="6">
-        <f>3+1+5</f>
-        <v>9</v>
+        <f>2+1+5</f>
+        <v>8</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
@@ -2157,7 +2155,7 @@
         <v>62</v>
       </c>
       <c r="B27" s="6">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="C27" s="6">
         <v>130</v>
@@ -2165,8 +2163,8 @@
       <c r="D27" s="6">
         <v>31</v>
       </c>
-      <c r="E27" s="6" t="s">
-        <v>70</v>
+      <c r="E27" s="24" t="s">
+        <v>71</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>

</xml_diff>

<commit_message>
change Min Max VO2Max Change RHH Min
</commit_message>
<xml_diff>
--- a/Lab4_BVT.xlsx
+++ b/Lab4_BVT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\SQA\Lab4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0696BBE3-6B3F-4D41-900B-2E87911D6A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C53E3A14-422E-45B1-B354-047373D3979F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="1" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="4" r:id="rId1"/>
@@ -1481,6 +1481,10 @@
       <c r="M22" s="2"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="B23" s="1" t="str">
+        <f>"B9"</f>
+        <v>B9</v>
+      </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>

</xml_diff>

<commit_message>
Modified Actual Result, Defect in Lab4_BVT.xlsx
</commit_message>
<xml_diff>
--- a/Lab4_BVT.xlsx
+++ b/Lab4_BVT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\SQA\Lab4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C53E3A14-422E-45B1-B354-047373D3979F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62188C0B-2E0E-4538-90D6-57EA27F782D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="1" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{2D3B1ECF-CE0B-884D-A6E2-5EDB198A06FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Summary" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="80">
   <si>
     <t>Test Case Design and Test Results</t>
   </si>
@@ -245,16 +245,40 @@
     <t>ธนภูมิ แทนทุมมา</t>
   </si>
   <si>
-    <t>java 26.0.1 2026-04-21, window 11</t>
-  </si>
-  <si>
-    <t>ค่า VO2 Max ไม่อยู่ในขอบเขต</t>
-  </si>
-  <si>
-    <t>ค่า RHR ไม่อยู่ในขอบเขตค่าที่กำหนด</t>
-  </si>
-  <si>
-    <t>ค่า HRR ไม่อยู่ในขอบเขตค่าที่กำหนด</t>
+    <t>VO2Max Out of Index</t>
+  </si>
+  <si>
+    <t>RHR Out of Index</t>
+  </si>
+  <si>
+    <t>HRR Out of Index</t>
+  </si>
+  <si>
+    <t>Failed to convert String "VO2Max Out of Index" to type java.lang.Integer</t>
+  </si>
+  <si>
+    <t>Failed to convert String "RHR Out of Index" to type java.lang.Integer</t>
+  </si>
+  <si>
+    <t>Failed to convert String "HRR Out of Index" to type java.lang.Integer</t>
+  </si>
+  <si>
+    <t>DF1</t>
+  </si>
+  <si>
+    <t>แปลงค่า String เป็น integer ไม่ได้</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Middle</t>
+  </si>
+  <si>
+    <t>ไม่สามารถแปลงค่า String เป็น Integer ได้</t>
+  </si>
+  <si>
+    <t>java 26.0.1 2026-04-21, window 11, Eclipse2026-6</t>
   </si>
 </sst>
 </file>
@@ -512,6 +536,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -521,31 +546,30 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
@@ -923,8 +947,12 @@
       <c r="B3" s="3">
         <v>13</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="C3" s="3">
+        <v>13</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="17"/>
@@ -936,8 +964,12 @@
       <c r="B4" s="3">
         <v>19</v>
       </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
+      <c r="C4" s="6">
+        <v>14</v>
+      </c>
+      <c r="D4" s="6">
+        <v>5</v>
+      </c>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -958,8 +990,12 @@
       <c r="B6" s="3">
         <v>32</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="19"/>
+      <c r="C6" s="18">
+        <v>27</v>
+      </c>
+      <c r="D6" s="19">
+        <v>5</v>
+      </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="20"/>
@@ -987,15 +1023,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="28"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
         <v>63</v>
@@ -1026,12 +1062,12 @@
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
@@ -1055,12 +1091,12 @@
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1084,12 +1120,12 @@
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="30" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="32"/>
+      <c r="B5" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
@@ -1124,7 +1160,7 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="25.05" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="35" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="34" t="s">
@@ -1132,13 +1168,13 @@
       </c>
       <c r="C7" s="34"/>
       <c r="D7" s="34"/>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="35" t="s">
+      <c r="F7" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="36" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -1155,7 +1191,7 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A8" s="33"/>
+      <c r="A8" s="35"/>
       <c r="B8" s="8" t="s">
         <v>63</v>
       </c>
@@ -1165,9 +1201,9 @@
       <c r="D8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="36"/>
       <c r="J8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1198,8 +1234,12 @@
         <f>0+1+3</f>
         <v>4</v>
       </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+      <c r="F9" s="6">
+        <v>4</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A10" s="6" t="s">
@@ -1218,8 +1258,12 @@
         <f>0+1+3</f>
         <v>4</v>
       </c>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="F10" s="6">
+        <v>4</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A11" s="6" t="s">
@@ -1238,8 +1282,12 @@
         <f>2+1+3</f>
         <v>6</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="F11" s="6">
+        <v>6</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -1262,8 +1310,12 @@
         <f>4+1+3</f>
         <v>8</v>
       </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="F12" s="6">
+        <v>8</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -1286,8 +1338,12 @@
         <f>5+1+3</f>
         <v>9</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="F13" s="6">
+        <v>9</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -1310,8 +1366,12 @@
         <f>2+5+3</f>
         <v>10</v>
       </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+      <c r="F14" s="6">
+        <v>10</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -1334,8 +1394,12 @@
         <f>2+5+3</f>
         <v>10</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+      <c r="F15" s="6">
+        <v>10</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -1358,8 +1422,12 @@
         <f>2+1+3</f>
         <v>6</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
+      <c r="F16" s="6">
+        <v>6</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -1382,8 +1450,12 @@
         <f>2+1+3</f>
         <v>6</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
+      <c r="F17" s="6">
+        <v>6</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.75">
@@ -1403,8 +1475,12 @@
         <f>2+1+1</f>
         <v>4</v>
       </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="F18" s="6">
+        <v>4</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -1427,8 +1503,12 @@
         <f>2+1+1</f>
         <v>4</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="F19" s="6">
+        <v>4</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A20" s="6" t="s">
@@ -1447,8 +1527,12 @@
         <f>2+1+5</f>
         <v>8</v>
       </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
+      <c r="F20" s="6">
+        <v>8</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A21" s="6" t="s">
@@ -1467,8 +1551,12 @@
         <f>2+1+5</f>
         <v>8</v>
       </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
+      <c r="F21" s="6">
+        <v>8</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -1481,10 +1569,6 @@
       <c r="M22" s="2"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="B23" s="1" t="str">
-        <f>"B9"</f>
-        <v>B9</v>
-      </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -1541,7 +1625,7 @@
     <col min="1" max="1" width="19.796875" style="1" customWidth="1"/>
     <col min="2" max="4" width="21.296875" style="1" customWidth="1"/>
     <col min="5" max="5" width="45.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.19921875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="67.69921875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.19921875" style="1" customWidth="1"/>
     <col min="8" max="10" width="10.796875" style="1"/>
     <col min="11" max="11" width="15.296875" style="1" customWidth="1"/>
@@ -1551,15 +1635,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="28"/>
       <c r="J1" s="2"/>
       <c r="K1" s="8" t="s">
         <v>63</v>
@@ -1590,12 +1674,12 @@
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
       <c r="F3" s="5" t="s">
         <v>21</v>
       </c>
@@ -1619,12 +1703,12 @@
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
       <c r="F4" s="5" t="s">
         <v>3</v>
       </c>
@@ -1648,12 +1732,12 @@
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="30" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="32"/>
+      <c r="B5" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="31"/>
       <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
@@ -1688,7 +1772,7 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="25.05" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="35" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="34" t="s">
@@ -1696,13 +1780,13 @@
       </c>
       <c r="C7" s="34"/>
       <c r="D7" s="34"/>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="35" t="s">
+      <c r="F7" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="36" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -1719,7 +1803,7 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A8" s="33"/>
+      <c r="A8" s="35"/>
       <c r="B8" s="8" t="s">
         <v>63</v>
       </c>
@@ -1729,9 +1813,9 @@
       <c r="D8" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="36"/>
       <c r="J8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1758,11 +1842,15 @@
       <c r="D9" s="6">
         <v>15</v>
       </c>
-      <c r="E9" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+      <c r="E9" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A10" s="6" t="s">
@@ -1781,8 +1869,12 @@
         <f>0+1+3</f>
         <v>4</v>
       </c>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="F10" s="6">
+        <v>4</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A11" s="6" t="s">
@@ -1801,8 +1893,12 @@
         <f>0+1+3</f>
         <v>4</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="F11" s="6">
+        <v>4</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
@@ -1825,8 +1921,12 @@
         <f>2+1+3</f>
         <v>6</v>
       </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="F12" s="6">
+        <v>6</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
@@ -1849,8 +1949,12 @@
         <f>4+1+3</f>
         <v>8</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="F13" s="6">
+        <v>8</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
@@ -1873,8 +1977,12 @@
         <f>5+1+3</f>
         <v>9</v>
       </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+      <c r="F14" s="6">
+        <v>9</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
@@ -1897,8 +2005,12 @@
         <f>5+1+3</f>
         <v>9</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+      <c r="F15" s="6">
+        <v>9</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
@@ -1918,10 +2030,14 @@
         <v>15</v>
       </c>
       <c r="E16" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
+        <v>69</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
@@ -1944,8 +2060,12 @@
         <f>2+5+3</f>
         <v>10</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
+      <c r="F17" s="6">
+        <v>10</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J17" s="2"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.75">
@@ -1965,8 +2085,12 @@
         <f>2+5+3</f>
         <v>10</v>
       </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="F18" s="6">
+        <v>10</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
@@ -1989,8 +2113,12 @@
         <f>2+1+3</f>
         <v>6</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="F19" s="6">
+        <v>6</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A20" s="6" t="s">
@@ -2009,8 +2137,12 @@
         <f>2+1+3</f>
         <v>6</v>
       </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
+      <c r="F20" s="6">
+        <v>6</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.75">
       <c r="A21" s="22" t="s">
@@ -2026,10 +2158,14 @@
         <v>15</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
+        <v>69</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -2049,10 +2185,14 @@
         <v>-1</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -2075,8 +2215,12 @@
         <f>2+1+1</f>
         <v>4</v>
       </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
+      <c r="F23" s="6">
+        <v>4</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -2099,8 +2243,12 @@
         <f>2+1+1</f>
         <v>4</v>
       </c>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
+      <c r="F24" s="6">
+        <v>4</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
@@ -2123,8 +2271,12 @@
         <f>2+1+5</f>
         <v>8</v>
       </c>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
+      <c r="F25" s="6">
+        <v>8</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
@@ -2147,8 +2299,12 @@
         <f>2+1+5</f>
         <v>8</v>
       </c>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
+      <c r="F26" s="6">
+        <v>8</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
@@ -2168,10 +2324,14 @@
         <v>31</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.75">
@@ -2201,7 +2361,13 @@
   <dimension ref="A2:K3"/>
   <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="27" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="16384" width="10.796875" style="1"/>
+    <col min="1" max="2" width="10.796875" style="1"/>
+    <col min="3" max="3" width="37.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.796875" style="1"/>
+    <col min="6" max="6" width="22.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="10" width="10.796875" style="1"/>
+    <col min="11" max="11" width="47.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="10.796875" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:11" ht="54" x14ac:dyDescent="0.75">
@@ -2243,16 +2409,32 @@
       <c r="A3" s="11">
         <v>1</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="12"/>
+      <c r="B3" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="12">
+        <v>46220</v>
+      </c>
       <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
+      <c r="F3" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="11">
+        <v>1</v>
+      </c>
       <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
+      <c r="K3" s="11" t="s">
+        <v>78</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>